<commit_message>
Append ten source-reviewed UESTC profiles and conserve existing department members
</commit_message>
<xml_diff>
--- a/site/exports/uestc-applied-math-center.xlsx
+++ b/site/exports/uestc-applied-math-center.xlsx
@@ -14,11 +14,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'总览'!$A$1:$K$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'经历'!$A$1:$S$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'总览'!$A$1:$K$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'经历'!$A$1:$S$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'导师'!$A$1:$L$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'论文'!$A$1:$L$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'来源'!$A$1:$G$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'论文'!$A$1:$L$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'来源'!$A$1:$G$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -675,10 +675,64 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>周冠宇</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>校区未标注</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>应用数学中心</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>https://faculty.uestc.edu.cn/zhouguanyu/zh_CN/index/358915/list/index.htm</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>本科、硕士教育未列；博士专业、入学时间、明确授位月日及法律授位主体未知。；自身导师、博士论文及论文导师未知；博士生导师是本人资格，不是自身导师。；工作经历数学科学院标签不自动纠正或合并组织；目录应用数学中心不证明行政隶属或当前在岗。；两篇作品通讯/贡献角色未知，外部出版元数据与全文未核；列首位仅反映原作者顺序。；页面最后更新时间与观察日实时人事状态未知。；当前人事状态未核，原岗位历史状态保持，不启用现职导航。；本人导师与原论文未核，不从博导资格推本人的师承。；院校985及地域分类未独立规范化，保持unknown。</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>分批核实资料，不是完整名录；人物整体核验日期未单独记录</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>公开个人页（访问与内容时效见来源记录）</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>uestc</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>电子科技大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K4"/>
+  <autoFilter ref="A1:K5"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -690,7 +744,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S20"/>
+  <dimension ref="A1:S24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2098,8 +2152,244 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>周冠宇</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>degree</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>博士</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>东京大学</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr"/>
+      <c r="F21" s="2" t="inlineStr"/>
+      <c r="G21" s="2" t="inlineStr"/>
+      <c r="H21" s="2" t="inlineStr"/>
+      <c r="I21" s="2" t="inlineStr"/>
+      <c r="J21" s="2" t="inlineStr"/>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M21" s="2" t="inlineStr"/>
+      <c r="N21" s="2" t="inlineStr"/>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>明确获授与年份；不由任教学科补博士专业，不补本硕教育或原论文导师。来源明确授位年份：2015。</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="inlineStr"/>
+      <c r="Q21" s="3" t="inlineStr">
+        <is>
+          <t>https://faculty.uestc.edu.cn/zhouguanyu/zh_CN/index/358915/list/index.htm</t>
+        </is>
+      </c>
+      <c r="R21" s="2" t="inlineStr">
+        <is>
+          <t>uestc</t>
+        </is>
+      </c>
+      <c r="S21" s="2" t="inlineStr">
+        <is>
+          <t>电子科技大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>周冠宇</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>postdoctoral</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>博士后</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>东京大学</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr"/>
+      <c r="H22" s="2" t="inlineStr"/>
+      <c r="I22" s="2" t="inlineStr"/>
+      <c r="J22" s="2" t="inlineStr"/>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="M22" s="2" t="inlineStr"/>
+      <c r="N22" s="2" t="inlineStr"/>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>博士后研究员工作为非学位经历，不新增博士获授。</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr"/>
+      <c r="Q22" s="3" t="inlineStr">
+        <is>
+          <t>https://faculty.uestc.edu.cn/zhouguanyu/zh_CN/index/358915/list/index.htm</t>
+        </is>
+      </c>
+      <c r="R22" s="2" t="inlineStr">
+        <is>
+          <t>uestc</t>
+        </is>
+      </c>
+      <c r="S22" s="2" t="inlineStr">
+        <is>
+          <t>电子科技大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>周冠宇</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>助理教授</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>东京理科大学</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr"/>
+      <c r="G23" s="2" t="inlineStr"/>
+      <c r="H23" s="2" t="inlineStr"/>
+      <c r="I23" s="2" t="inlineStr"/>
+      <c r="J23" s="2" t="inlineStr"/>
+      <c r="K23" s="2" t="inlineStr"/>
+      <c r="L23" s="2" t="inlineStr"/>
+      <c r="M23" s="2" t="inlineStr"/>
+      <c r="N23" s="2" t="inlineStr"/>
+      <c r="O23" s="2" t="inlineStr"/>
+      <c r="P23" s="2" t="inlineStr"/>
+      <c r="Q23" s="3" t="inlineStr">
+        <is>
+          <t>https://faculty.uestc.edu.cn/zhouguanyu/zh_CN/index/358915/list/index.htm</t>
+        </is>
+      </c>
+      <c r="R23" s="2" t="inlineStr">
+        <is>
+          <t>uestc</t>
+        </is>
+      </c>
+      <c r="S23" s="2" t="inlineStr">
+        <is>
+          <t>电子科技大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>周冠宇</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>教授</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>电子科技大学</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>2019-11</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr"/>
+      <c r="G24" s="2" t="inlineStr"/>
+      <c r="H24" s="2" t="inlineStr"/>
+      <c r="I24" s="2" t="inlineStr"/>
+      <c r="J24" s="2" t="inlineStr"/>
+      <c r="K24" s="2" t="inlineStr"/>
+      <c r="L24" s="2" t="inlineStr"/>
+      <c r="M24" s="2" t="inlineStr"/>
+      <c r="N24" s="2" t="inlineStr"/>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>个人简介另写2019年至今在基础与前沿研究院；任职主体标签分别保留，不推行政结构或实时在岗。</t>
+        </is>
+      </c>
+      <c r="P24" s="2" t="inlineStr"/>
+      <c r="Q24" s="3" t="inlineStr">
+        <is>
+          <t>https://faculty.uestc.edu.cn/zhouguanyu/zh_CN/index/358915/list/index.htm</t>
+        </is>
+      </c>
+      <c r="R24" s="2" t="inlineStr">
+        <is>
+          <t>uestc</t>
+        </is>
+      </c>
+      <c r="S24" s="2" t="inlineStr">
+        <is>
+          <t>电子科技大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S20"/>
+  <autoFilter ref="A1:S24"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -2120,6 +2410,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId23"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2401,7 +2695,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2409,7 +2703,7 @@
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="25.2" customWidth="1" min="4" max="4"/>
     <col width="65" customWidth="1" min="5" max="5"/>
-    <col width="29.4" customWidth="1" min="6" max="6"/>
+    <col width="51.8" customWidth="1" min="6" max="6"/>
     <col width="65" customWidth="1" min="7" max="7"/>
     <col width="65" customWidth="1" min="8" max="8"/>
     <col width="65" customWidth="1" min="9" max="9"/>
@@ -2764,8 +3058,120 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>周冠宇</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>An analysis on the finite volume schemes and the discrete Lyapunov inequalities for the chemotaxis system</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>2021</v>
+      </c>
+      <c r="D7" s="2" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>https://faculty.uestc.edu.cn/zhouguanyu/zh_CN/lwcg/358920/list/index.htm</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>期刊论文；journal_article_as_official_list</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>https://faculty.uestc.edu.cn/zhouguanyu/zh_CN/lwcg/358920/list/index.htm</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>https://faculty.uestc.edu.cn/zhouguanyu/zh_CN/lwcg/358920/list/index.htm</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>仅官网书目，未核外部元数据或全文。；official_publication_list_only</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>官网书目原作者、年份、期刊等直接对应；链接未打开，外部元数据与全文未知。</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>uestc</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>电子科技大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>周冠宇</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>An analysis on the penalty and Nitsche's methods for the Stokes-Darcy system with a curved interface</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>2021</v>
+      </c>
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>https://faculty.uestc.edu.cn/zhouguanyu/zh_CN/lwcg/358920/list/index.htm</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>期刊论文；journal_article_as_official_list</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>https://faculty.uestc.edu.cn/zhouguanyu/zh_CN/lwcg/358920/list/index.htm</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>https://faculty.uestc.edu.cn/zhouguanyu/zh_CN/lwcg/358920/list/index.htm</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>仅官网书目，未核外部元数据或全文。；official_publication_list_only</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>官网书目原作者、年份、期刊等直接对应；链接未打开，外部元数据与全文未知。</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>uestc</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>电子科技大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L6"/>
+  <autoFilter ref="A1:L8"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId2"/>
@@ -2782,6 +3188,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId21"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2793,11 +3205,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="39.2" customWidth="1" min="2" max="2"/>
+    <col width="49" customWidth="1" min="2" max="2"/>
     <col width="65" customWidth="1" min="3" max="3"/>
     <col width="65" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
@@ -3400,27 +3812,27 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>顾亦奇</t>
+          <t>周冠宇</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>institution-classification-8</t>
+          <t>uestc-zhouguanyu-profile</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>https://www.moe.gov.cn/srcsite/A22/s7065/200612/t20061206_128833.html</t>
+          <t>https://faculty.uestc.edu.cn/zhouguanyu/zh_CN/index/358915/list/index.htm</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>历史985院校分类参考；非个人授位或就读当年建设身份的证明</t>
+          <t>official_public_body_read</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>未单独记录</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -3437,42 +3849,153 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
+          <t>周冠宇</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>uestc-zhouguanyu-bibliography</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>https://faculty.uestc.edu.cn/zhouguanyu/zh_CN/lwcg/358920/list/index.htm</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>official_public_body_read</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>uestc</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>电子科技大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>周冠宇</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>uestc-applied-mathematics-directory</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>https://cam.uestc.edu.cn/szdw/jzry.htm</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>official_public_body_read</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>uestc</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>电子科技大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>顾亦奇</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>institution-classification-8</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>https://www.moe.gov.cn/srcsite/A22/s7065/200612/t20061206_128833.html</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>历史985院校分类参考；非个人授位或就读当年建设身份的证明</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>未单独记录</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>uestc</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>电子科技大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
           <t>孔婀芳</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>institution-classification-3</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr">
         <is>
           <t>https://www.moe.gov.cn/srcsite/A22/s7065/200612/t20061206_128833.html</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>历史985院校分类参考；非个人授位或就读当年建设身份的证明</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>未单独记录</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>uestc</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>uestc</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
         <is>
           <t>电子科技大学</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G18"/>
+  <autoFilter ref="A1:G21"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
@@ -3491,6 +4014,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId20"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>